<commit_message>
Revised task 3 and begin task 4, remove the year to avoid overlap
</commit_message>
<xml_diff>
--- a/data/Original_UICLibraryData.xlsx
+++ b/data/Original_UICLibraryData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Henry\Downloads\CS424_P1\Project-1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Henry\Downloads\CS424_P1\Project-1\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9849FB23-40FF-4535-B94D-16D145BEE4AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F7485C1-CDBA-4A62-B553-47A708EA947D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{68D7DA14-3BBB-4245-B58F-0CCF1E067232}"/>
   </bookViews>
@@ -77,21 +77,6 @@
     <t>floor</t>
   </si>
   <si>
-    <t>9/21/2026</t>
-  </si>
-  <si>
-    <t>9/22/2026</t>
-  </si>
-  <si>
-    <t>9/24/2026</t>
-  </si>
-  <si>
-    <t>9/25/2026</t>
-  </si>
-  <si>
-    <t>9/23/2026</t>
-  </si>
-  <si>
     <t>53</t>
   </si>
   <si>
@@ -126,6 +111,21 @@
   </si>
   <si>
     <t>second</t>
+  </si>
+  <si>
+    <t>9/21</t>
+  </si>
+  <si>
+    <t>9/22</t>
+  </si>
+  <si>
+    <t>9/23</t>
+  </si>
+  <si>
+    <t>9/24</t>
+  </si>
+  <si>
+    <t>9/25</t>
   </si>
 </sst>
 </file>
@@ -530,16 +530,16 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="E2" t="s">
         <v>1</v>
@@ -547,16 +547,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s">
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
         <v>3</v>
@@ -567,16 +567,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
         <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E4" t="s">
         <v>1</v>
@@ -584,16 +584,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
         <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E5" t="s">
         <v>3</v>
@@ -604,16 +604,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="B6" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="E6" t="s">
         <v>1</v>
@@ -621,16 +621,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
         <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E7" t="s">
         <v>3</v>
@@ -641,16 +641,16 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
         <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E8" t="s">
         <v>1</v>
@@ -658,16 +658,16 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s">
         <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s">
         <v>2</v>
@@ -678,16 +678,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
         <v>0</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E10" t="s">
         <v>1</v>
@@ -698,16 +698,16 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
         <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
         <v>2</v>

</xml_diff>